<commit_message>
Correct eight points in Confidence Intervals for a Mean
The t-interval is wider than the z-formula for the same s and wider on average, but s can land below sigma, so the challenge hint and quiz no longer promise a wider interval every time. The conditions now include independence, and the z-interval is exact for normal data. The figure draws the normal and t (3 df) from their densities. The delivery interval is give or take an hour and a half and describes the average shipment, the AI table uses independent seeds rather than correlated folds, comparisons use an interval on the difference, and the data is a realistic teaching set.
</commit_message>
<xml_diff>
--- a/data/confidence-intervals-for-a-mean--delivery_times.xlsx
+++ b/data/confidence-intervals-for-a-mean--delivery_times.xlsx
@@ -5711,7 +5711,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WHAT IS CAPTURED: completed shipment records from a logistics system.</t>
+          <t>WHAT IS CAPTURED: completed shipment records from a logistics system (a realistic teaching dataset written for the book).</t>
         </is>
       </c>
     </row>
@@ -5725,7 +5725,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Check conditions: roughly symmetric / large enough n for the CLT.</t>
+          <t>Check conditions: independent shipments, and roughly symmetric data or a large enough n for the CLT.</t>
         </is>
       </c>
     </row>

</xml_diff>